<commit_message>
Close pre-launch audit gaps: breach coverage, policy-ID sync, CI checks
</commit_message>
<xml_diff>
--- a/templates/ropa/ROPA-template.xlsx
+++ b/templates/ropa/ROPA-template.xlsx
@@ -24,10 +24,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
   <si>
-    <t xml:space="preserve">ROPA — Register Information</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not legal advice. Synthetic data only — never enter real records.</t>
+    <t xml:space="preserve">ROPA - Register Information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not legal advice. Synthetic data only - never enter real records.</t>
   </si>
   <si>
     <t xml:space="preserve">Organisation (controller)</t>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">Legitimate interests</t>
   </si>
   <si>
-    <t xml:space="preserve">Record of Processing Activities — one row per activity</t>
+    <t xml:space="preserve">Record of Processing Activities - one row per activity</t>
   </si>
   <si>
     <t xml:space="preserve">Fill one row per processing activity. Tier pulls from the Classification Matrix. Yellow = to complete.</t>

</xml_diff>